<commit_message>
Update test spreadsheets with latest E2E runs and static security audit outputs
</commit_message>
<xml_diff>
--- a/selenium-tests/test_report.xlsx
+++ b/selenium-tests/test_report.xlsx
@@ -29,7 +29,7 @@
     <t>Test Execution Date</t>
   </si>
   <si>
-    <t>15/6/2026, 1:15:43 pm</t>
+    <t>15/6/2026, 1:50:09 pm</t>
   </si>
   <si>
     <t>Total Steps Executed</t>
@@ -74,7 +74,7 @@
     <t>PASSED</t>
   </si>
   <si>
-    <t>2026-06-15T07:45:27.579Z</t>
+    <t>2026-06-15T08:19:55.774Z</t>
   </si>
   <si>
     <t>Static server hosted successfully</t>
@@ -83,7 +83,7 @@
     <t>WebDriver Session Initialization</t>
   </si>
   <si>
-    <t>2026-06-15T07:45:32.795Z</t>
+    <t>2026-06-15T08:19:57.804Z</t>
   </si>
   <si>
     <t>Chrome headless instance created</t>
@@ -92,7 +92,7 @@
     <t>Load Application URL</t>
   </si>
   <si>
-    <t>2026-06-15T07:45:33.186Z</t>
+    <t>2026-06-15T08:19:59.217Z</t>
   </si>
   <si>
     <t>Target loaded at http://localhost:8095</t>
@@ -101,7 +101,7 @@
     <t>Check Flutter Canvas Elements</t>
   </si>
   <si>
-    <t>2026-06-15T07:45:34.304Z</t>
+    <t>2026-06-15T08:20:00.340Z</t>
   </si>
   <si>
     <t>Glass pane initialized in DOM</t>
@@ -110,7 +110,7 @@
     <t>Enable Web Accessibility Semantics</t>
   </si>
   <si>
-    <t>2026-06-15T07:45:34.315Z</t>
+    <t>2026-06-15T08:20:00.561Z</t>
   </si>
   <si>
     <t>Accessibility tree configured: SUCCESS</t>
@@ -119,7 +119,7 @@
     <t>Verify Slide 1: Welcome Screen Text</t>
   </si>
   <si>
-    <t>2026-06-15T07:45:38.591Z</t>
+    <t>2026-06-15T08:20:03.836Z</t>
   </si>
   <si>
     <t>Main onboarding welcome text verified</t>
@@ -128,7 +128,7 @@
     <t>Verify Onboarding Pagination Dots</t>
   </si>
   <si>
-    <t>2026-06-15T07:45:38.624Z</t>
+    <t>2026-06-15T08:20:03.899Z</t>
   </si>
   <si>
     <t>Skip overlay controls are interactable</t>
@@ -137,7 +137,7 @@
     <t>Verify Skip Button Interactive Bounds</t>
   </si>
   <si>
-    <t>2026-06-15T07:45:38.640Z</t>
+    <t>2026-06-15T08:20:03.903Z</t>
   </si>
   <si>
     <t>Skip action element verified in semantics tree</t>
@@ -146,7 +146,7 @@
     <t>Perform Skip Redirection Transition</t>
   </si>
   <si>
-    <t>2026-06-15T07:45:39.016Z</t>
+    <t>2026-06-15T08:20:04.368Z</t>
   </si>
   <si>
     <t>Redirection to auth screen verified</t>
@@ -155,7 +155,7 @@
     <t>Verify Sign In Heading Presence</t>
   </si>
   <si>
-    <t>2026-06-15T07:45:39.035Z</t>
+    <t>2026-06-15T08:20:04.408Z</t>
   </si>
   <si>
     <t>Login branding header located</t>
@@ -164,7 +164,7 @@
     <t>Submit Blank Form to Verify Inputs</t>
   </si>
   <si>
-    <t>2026-06-15T07:45:40.084Z</t>
+    <t>2026-06-15T08:20:05.441Z</t>
   </si>
   <si>
     <t>Submitted empty credentials form</t>
@@ -173,7 +173,7 @@
     <t>Check Validation Warn: Email Missing</t>
   </si>
   <si>
-    <t>2026-06-15T07:45:40.090Z</t>
+    <t>2026-06-15T08:20:05.460Z</t>
   </si>
   <si>
     <t>Blank validation triggers correct warning</t>
@@ -182,7 +182,7 @@
     <t>Inject Malformed Username Format</t>
   </si>
   <si>
-    <t>2026-06-15T07:45:40.102Z</t>
+    <t>2026-06-15T08:20:05.479Z</t>
   </si>
   <si>
     <t>Typed invalid format string</t>
@@ -191,7 +191,7 @@
     <t>Submit Credentials Payload</t>
   </si>
   <si>
-    <t>2026-06-15T07:45:43.149Z</t>
+    <t>2026-06-15T08:20:08.628Z</t>
   </si>
   <si>
     <t>Dispatched validation credentials</t>
@@ -200,7 +200,7 @@
     <t>Shutdown Browser &amp; Terminate Server</t>
   </si>
   <si>
-    <t>2026-06-15T07:45:43.458Z</t>
+    <t>2026-06-15T08:20:09.054Z</t>
   </si>
   <si>
     <t>All background processes killed cleanly</t>
@@ -703,7 +703,7 @@
         <v>11</v>
       </c>
       <c r="B8" s="3">
-        <v>17.91</v>
+        <v>15.95</v>
       </c>
     </row>
   </sheetData>
@@ -755,7 +755,7 @@
         <v>19</v>
       </c>
       <c r="D2" s="9">
-        <v>2036</v>
+        <v>2672</v>
       </c>
       <c r="E2" t="s">
         <v>20</v>
@@ -775,7 +775,7 @@
         <v>19</v>
       </c>
       <c r="D3" s="9">
-        <v>5216</v>
+        <v>2030</v>
       </c>
       <c r="E3" t="s">
         <v>23</v>
@@ -795,7 +795,7 @@
         <v>19</v>
       </c>
       <c r="D4" s="9">
-        <v>391</v>
+        <v>1413</v>
       </c>
       <c r="E4" t="s">
         <v>26</v>
@@ -815,7 +815,7 @@
         <v>19</v>
       </c>
       <c r="D5" s="9">
-        <v>1118</v>
+        <v>1123</v>
       </c>
       <c r="E5" t="s">
         <v>29</v>
@@ -835,7 +835,7 @@
         <v>19</v>
       </c>
       <c r="D6" s="9">
-        <v>10</v>
+        <v>221</v>
       </c>
       <c r="E6" t="s">
         <v>32</v>
@@ -855,7 +855,7 @@
         <v>19</v>
       </c>
       <c r="D7" s="9">
-        <v>4276</v>
+        <v>3275</v>
       </c>
       <c r="E7" t="s">
         <v>35</v>
@@ -875,7 +875,7 @@
         <v>19</v>
       </c>
       <c r="D8" s="9">
-        <v>33</v>
+        <v>63</v>
       </c>
       <c r="E8" t="s">
         <v>38</v>
@@ -895,7 +895,7 @@
         <v>19</v>
       </c>
       <c r="D9" s="9">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E9" t="s">
         <v>41</v>
@@ -915,7 +915,7 @@
         <v>19</v>
       </c>
       <c r="D10" s="9">
-        <v>376</v>
+        <v>465</v>
       </c>
       <c r="E10" t="s">
         <v>44</v>
@@ -935,7 +935,7 @@
         <v>19</v>
       </c>
       <c r="D11" s="9">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="E11" t="s">
         <v>47</v>
@@ -955,7 +955,7 @@
         <v>19</v>
       </c>
       <c r="D12" s="9">
-        <v>1049</v>
+        <v>1033</v>
       </c>
       <c r="E12" t="s">
         <v>50</v>
@@ -975,7 +975,7 @@
         <v>19</v>
       </c>
       <c r="D13" s="9">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="E13" t="s">
         <v>53</v>
@@ -995,7 +995,7 @@
         <v>19</v>
       </c>
       <c r="D14" s="9">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E14" t="s">
         <v>56</v>
@@ -1015,7 +1015,7 @@
         <v>19</v>
       </c>
       <c r="D15" s="9">
-        <v>3047</v>
+        <v>3148</v>
       </c>
       <c r="E15" t="s">
         <v>59</v>
@@ -1035,7 +1035,7 @@
         <v>19</v>
       </c>
       <c r="D16" s="9">
-        <v>309</v>
+        <v>425</v>
       </c>
       <c r="E16" t="s">
         <v>62</v>

</xml_diff>